<commit_message>
Update modeling analysis, results, and documentation
</commit_message>
<xml_diff>
--- a/results/result1.xlsx
+++ b/results/result1.xlsx
@@ -1984,7 +1984,7 @@
         <v>833.333333</v>
       </c>
       <c r="C3" t="n">
-        <v>6365.841099</v>
+        <v>5947.419649</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -2002,10 +2002,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4787.964164</v>
+        <v>3954.63083</v>
       </c>
       <c r="C4" t="n">
-        <v>1702.996983</v>
+        <v>2121.418433</v>
       </c>
     </row>
     <row r="5" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5286.035177</v>
+        <v>6119.36851</v>
       </c>
       <c r="C5" t="n">
         <v>91.101383</v>
@@ -2031,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>5780.131883</v>
+        <v>5068.68685</v>
       </c>
     </row>
     <row r="7" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2044,7 +2044,7 @@
         <v>5333.333333</v>
       </c>
       <c r="C7" t="n">
-        <v>2859.868117</v>
+        <v>3571.31315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>